<commit_message>
Finalize launch surfaces and live voice policy
</commit_message>
<xml_diff>
--- a/output/spreadsheet/phrase_catalog_sorted.xlsx
+++ b/output/spreadsheet/phrase_catalog_sorted.xlsx
@@ -2253,12 +2253,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>15!</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>15!</t>
+          <t>15</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2454,12 +2454,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Go!</t>
+          <t>Go</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Kjør på nå.</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3884,8 +3884,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr">
         <is>
           <t>legacy HR correction variant</t>
@@ -3943,8 +3941,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr">
         <is>
           <t>legacy sustained HR correction variant</t>
@@ -4002,8 +3998,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
           <t>legacy sustained HR correction variant</t>
@@ -4061,8 +4055,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
         <is>
           <t>legacy HR correction variant</t>
@@ -4120,8 +4112,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr">
         <is>
           <t>legacy sustained HR push variant</t>
@@ -4179,8 +4169,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
           <t>legacy sustained HR push variant</t>
@@ -4238,8 +4226,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr">
         <is>
           <t>legacy breath guidance</t>
@@ -4297,8 +4283,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr">
         <is>
           <t>legacy breath guidance</t>
@@ -4356,8 +4340,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr">
         <is>
           <t>legacy breath guidance</t>
@@ -4415,8 +4397,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr">
         <is>
           <t>legacy breath guidance</t>
@@ -4474,8 +4454,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr">
         <is>
           <t>legacy no-HR feel guidance</t>
@@ -4533,8 +4511,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr">
         <is>
           <t>legacy no-HR feel guidance</t>
@@ -4592,8 +4568,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr">
         <is>
           <t>legacy no-HR feel guidance</t>
@@ -4651,8 +4625,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr">
         <is>
           <t>legacy no-HR feel guidance</t>
@@ -4710,8 +4682,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr">
         <is>
           <t>legacy no-HR feel guidance</t>
@@ -4769,8 +4739,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr">
         <is>
           <t>legacy no-HR feel guidance</t>
@@ -4828,8 +4796,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr">
         <is>
           <t>legacy no-HR feel guidance</t>
@@ -4887,8 +4853,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr">
         <is>
           <t>legacy HR hold variant</t>
@@ -4946,8 +4910,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr">
         <is>
           <t>legacy flat motivation pool</t>
@@ -5005,8 +4967,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr">
         <is>
           <t>legacy flat motivation pool</t>
@@ -5064,8 +5024,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr">
         <is>
           <t>legacy flat motivation pool</t>
@@ -5123,8 +5081,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr">
         <is>
           <t>legacy flat motivation pool</t>
@@ -5182,8 +5138,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr">
         <is>
           <t>legacy flat motivation pool</t>
@@ -5241,8 +5195,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr">
         <is>
           <t>legacy flat motivation pool</t>
@@ -5300,8 +5252,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr">
         <is>
           <t>legacy flat motivation pool</t>
@@ -5359,8 +5309,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr">
         <is>
           <t>legacy flat motivation pool</t>
@@ -5418,8 +5366,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr">
         <is>
           <t>legacy flat motivation pool</t>
@@ -5477,8 +5423,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr">
         <is>
           <t>legacy flat motivation pool</t>
@@ -5536,8 +5480,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr">
         <is>
           <t>future HR-loss variant</t>
@@ -5595,8 +5537,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr">
         <is>
           <t>future HR-restore variant</t>
@@ -5654,8 +5594,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr">
         <is>
           <t>future no-HR mode-switch variant</t>
@@ -5713,8 +5651,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr">
         <is>
           <t>future shared main-set variant</t>
@@ -5772,8 +5708,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr">
         <is>
           <t>future shared main-set variant</t>
@@ -5831,8 +5765,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr">
         <is>
           <t>future pause-detected variant</t>
@@ -5890,8 +5822,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr"/>
-      <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr">
         <is>
           <t>future pause-resumed variant</t>
@@ -5949,8 +5879,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
         <is>
           <t>future shared cooldown variant</t>
@@ -6008,8 +5936,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr">
         <is>
           <t>future shared cooldown variant</t>
@@ -6067,8 +5993,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr"/>
-      <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr">
         <is>
           <t>future shared recovery variant</t>
@@ -6126,8 +6050,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr">
         <is>
           <t>future shared recovery variant</t>
@@ -6185,8 +6107,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr">
         <is>
           <t>future shared warmup variant</t>
@@ -6244,8 +6164,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr">
         <is>
           <t>future shared warmup variant</t>
@@ -6303,8 +6221,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr">
         <is>
           <t>future HR correction variant</t>
@@ -6362,8 +6278,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr">
         <is>
           <t>future HR correction variant</t>
@@ -6421,8 +6335,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr">
         <is>
           <t>future HR correction variant</t>
@@ -6480,8 +6392,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr">
         <is>
           <t>future HR correction variant</t>
@@ -6539,8 +6449,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr">
         <is>
           <t>future HR correction variant</t>
@@ -6598,8 +6506,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr">
         <is>
           <t>future HR correction variant</t>
@@ -6657,8 +6563,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr">
         <is>
           <t>future HR correction variant</t>
@@ -6716,8 +6620,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr">
         <is>
           <t>future HR correction variant</t>
@@ -6775,8 +6677,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr">
         <is>
           <t>future HR hold variant</t>
@@ -6834,8 +6734,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr">
         <is>
           <t>future HR hold variant</t>
@@ -6893,8 +6791,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr">
         <is>
           <t>future HR hold variant</t>
@@ -6952,8 +6848,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr">
         <is>
           <t>future HR hold variant</t>
@@ -7011,8 +6905,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
           <t>future easy-run motivation variant</t>
@@ -7070,8 +6962,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
           <t>future easy-run motivation variant</t>
@@ -7129,8 +7019,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
           <t>future easy-run motivation variant</t>
@@ -7188,8 +7076,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
           <t>future easy-run motivation variant</t>
@@ -7247,8 +7133,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr">
         <is>
           <t>future interval motivation variant</t>
@@ -7306,8 +7190,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
           <t>future interval motivation variant</t>
@@ -7365,8 +7247,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
           <t>future interval motivation variant</t>
@@ -7424,8 +7304,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
           <t>future interval motivation variant</t>
@@ -7483,8 +7361,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
           <t>future countdown-start variant</t>
@@ -7542,8 +7418,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr"/>
-      <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
           <t>future workout-finish variant</t>
@@ -7601,8 +7475,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="K115" t="inlineStr"/>
-      <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
           <t>future workout-finish variant</t>

</xml_diff>